<commit_message>
chore: 시험 진척도 갱신 (feature/tracker-pages, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -12294,7 +12294,7 @@
     <row r="6">
       <c r="A6" s="33" t="inlineStr">
         <is>
-          <t>2026-10-03 02:17</t>
+          <t>2026-10-03 02:22</t>
         </is>
       </c>
       <c r="B6" s="34" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="C6" s="33" t="inlineStr">
         <is>
-          <t>db9d588</t>
+          <t>cdc5392</t>
         </is>
       </c>
       <c r="D6" s="35" t="n">
@@ -12326,7 +12326,7 @@
         <v>260</v>
       </c>
       <c r="J6" s="35" t="n">
-        <v>14.5</v>
+        <v>17.8</v>
       </c>
       <c r="K6" s="36">
         <f>IFERROR(E6/(E6+F6+G6),0)</f>

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/sc02-dashboard, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$7</f>
+              <f>'실행이력'!$A$4:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$7</f>
+              <f>'실행이력'!$E$4:$E$8</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$7</f>
+              <f>'실행이력'!$A$4:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$7</f>
+              <f>'실행이력'!$F$4:$F$8</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$7</f>
+              <f>'실행이력'!$A$4:$A$8</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$7</f>
+              <f>'실행이력'!$G$4:$G$8</f>
             </numRef>
           </val>
         </ser>
@@ -9866,13 +9866,13 @@
         <v/>
       </c>
       <c r="D7" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="23" t="n">
         <v>0</v>
@@ -9894,13 +9894,13 @@
         <v/>
       </c>
       <c r="D8" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8" s="23" t="n">
         <v>0</v>
@@ -9922,13 +9922,13 @@
         <v/>
       </c>
       <c r="D9" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" s="23" t="n">
         <v>0</v>
@@ -9950,13 +9950,13 @@
         <v/>
       </c>
       <c r="D10" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="23" t="n">
         <v>0</v>
@@ -10874,13 +10874,13 @@
         <v/>
       </c>
       <c r="D43" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F43" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" s="23" t="n">
         <v>0</v>
@@ -10902,13 +10902,13 @@
         <v/>
       </c>
       <c r="D44" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F44" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44" s="23" t="n">
         <v>0</v>
@@ -10930,13 +10930,13 @@
         <v/>
       </c>
       <c r="D45" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="23" t="n">
         <v>0</v>
@@ -10958,13 +10958,13 @@
         <v/>
       </c>
       <c r="D46" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46" s="23" t="n">
         <v>0</v>
@@ -10986,13 +10986,13 @@
         <v/>
       </c>
       <c r="D47" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47" s="23" t="n">
         <v>0</v>
@@ -11014,13 +11014,13 @@
         <v/>
       </c>
       <c r="D48" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F48" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G48" s="23" t="n">
         <v>0</v>
@@ -11042,13 +11042,13 @@
         <v/>
       </c>
       <c r="D49" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E49" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G49" s="23" t="n">
         <v>0</v>
@@ -11070,13 +11070,13 @@
         <v/>
       </c>
       <c r="D50" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E50" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F50" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="23" t="n">
         <v>0</v>
@@ -12918,13 +12918,13 @@
         <v/>
       </c>
       <c r="D116" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E116" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F116" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G116" s="23" t="n">
         <v>0</v>
@@ -12946,13 +12946,13 @@
         <v/>
       </c>
       <c r="D117" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E117" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F117" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G117" s="23" t="n">
         <v>0</v>
@@ -12974,13 +12974,13 @@
         <v/>
       </c>
       <c r="D118" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E118" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F118" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G118" s="23" t="n">
         <v>0</v>
@@ -13002,13 +13002,13 @@
         <v/>
       </c>
       <c r="D119" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E119" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F119" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G119" s="23" t="n">
         <v>0</v>
@@ -13030,13 +13030,13 @@
         <v/>
       </c>
       <c r="D120" s="23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E120" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F120" s="23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G120" s="23" t="n">
         <v>0</v>
@@ -13058,13 +13058,13 @@
         <v/>
       </c>
       <c r="D121" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E121" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F121" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G121" s="23" t="n">
         <v>0</v>
@@ -13086,13 +13086,13 @@
         <v/>
       </c>
       <c r="D122" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E122" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F122" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G122" s="23" t="n">
         <v>0</v>
@@ -13114,13 +13114,13 @@
         <v/>
       </c>
       <c r="D123" s="23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E123" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F123" s="23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G123" s="23" t="n">
         <v>0</v>
@@ -13142,13 +13142,13 @@
         <v/>
       </c>
       <c r="D124" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E124" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F124" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124" s="23" t="n">
         <v>0</v>
@@ -13170,13 +13170,13 @@
         <v/>
       </c>
       <c r="D125" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E125" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F125" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G125" s="23" t="n">
         <v>0</v>
@@ -13198,13 +13198,13 @@
         <v/>
       </c>
       <c r="D126" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E126" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F126" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G126" s="23" t="n">
         <v>0</v>
@@ -13226,13 +13226,13 @@
         <v/>
       </c>
       <c r="D127" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E127" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F127" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G127" s="23" t="n">
         <v>0</v>
@@ -13254,13 +13254,13 @@
         <v/>
       </c>
       <c r="D128" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E128" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F128" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G128" s="23" t="n">
         <v>0</v>
@@ -13282,13 +13282,13 @@
         <v/>
       </c>
       <c r="D129" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E129" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F129" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G129" s="23" t="n">
         <v>0</v>
@@ -13310,13 +13310,13 @@
         <v/>
       </c>
       <c r="D130" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E130" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F130" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G130" s="23" t="n">
         <v>0</v>
@@ -13338,13 +13338,13 @@
         <v/>
       </c>
       <c r="D131" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E131" s="23" t="n">
         <v>0</v>
       </c>
       <c r="F131" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G131" s="23" t="n">
         <v>0</v>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14475,6 +14475,48 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-03 02:46</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t>feature/sc02-dashboard</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>ebf33d6</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E8" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F8" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G8" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="35" t="n">
+        <v>292</v>
+      </c>
+      <c r="J8" s="35" t="n">
+        <v>18</v>
+      </c>
+      <c r="K8" s="36">
+        <f>IFERROR(E8/(E8+F8+G8),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/sc02-screen-mapping, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$8</f>
+              <f>'실행이력'!$A$4:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$8</f>
+              <f>'실행이력'!$E$4:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$8</f>
+              <f>'실행이력'!$A$4:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$8</f>
+              <f>'실행이력'!$F$4:$F$9</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$8</f>
+              <f>'실행이력'!$A$4:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$8</f>
+              <f>'실행이력'!$G$4:$G$9</f>
             </numRef>
           </val>
         </ser>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="D8" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
@@ -2440,7 +2440,7 @@
       </c>
       <c r="D9" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="D10" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="D11" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="D44" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E44" s="27" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="D45" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="D46" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E46" s="27" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="D47" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E47" s="27" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="D48" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E48" s="27" t="inlineStr">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="D49" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E49" s="27" t="inlineStr">
@@ -4367,7 +4367,7 @@
       </c>
       <c r="D50" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E50" s="27" t="inlineStr">
@@ -4414,7 +4414,7 @@
       </c>
       <c r="D51" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr">
@@ -7516,7 +7516,7 @@
       </c>
       <c r="D117" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E117" s="27" t="inlineStr">
@@ -7563,7 +7563,7 @@
       </c>
       <c r="D118" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E118" s="27" t="inlineStr">
@@ -7610,7 +7610,7 @@
       </c>
       <c r="D119" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E119" s="27" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="D120" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E120" s="27" t="inlineStr">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="D121" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E121" s="27" t="inlineStr">
@@ -7751,7 +7751,7 @@
       </c>
       <c r="D122" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E122" s="27" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="D123" s="28" t="inlineStr">
         <is>
-          <t>SC-06</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E123" s="27" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="D124" s="28" t="inlineStr">
         <is>
-          <t>SC-03</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E124" s="27" t="inlineStr">
@@ -7892,7 +7892,7 @@
       </c>
       <c r="D125" s="28" t="inlineStr">
         <is>
-          <t>SC-07</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E125" s="27" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="D126" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E126" s="27" t="inlineStr">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="D127" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E127" s="27" t="inlineStr">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="D128" s="28" t="inlineStr">
         <is>
-          <t>SC-06</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E128" s="27" t="inlineStr">
@@ -8080,7 +8080,7 @@
       </c>
       <c r="D129" s="28" t="inlineStr">
         <is>
-          <t>SC-01</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E129" s="27" t="inlineStr">
@@ -8127,7 +8127,7 @@
       </c>
       <c r="D130" s="28" t="inlineStr">
         <is>
-          <t>SC-01</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E130" s="27" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="D131" s="28" t="inlineStr">
         <is>
-          <t>SC-01</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E131" s="27" t="inlineStr">
@@ -8221,7 +8221,7 @@
       </c>
       <c r="D132" s="28" t="inlineStr">
         <is>
-          <t>SC-04</t>
+          <t>SC-02</t>
         </is>
       </c>
       <c r="E132" s="27" t="inlineStr">
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14517,6 +14517,48 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-03 02:50</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>fix/sc02-screen-mapping</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>bc987b1</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F9" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="35" t="n">
+        <v>294</v>
+      </c>
+      <c r="J9" s="35" t="n">
+        <v>21</v>
+      </c>
+      <c r="K9" s="36">
+        <f>IFERROR(E9/(E9+F9+G9),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/tracker-cache-bust, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$9</f>
+              <f>'실행이력'!$A$4:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$9</f>
+              <f>'실행이력'!$E$4:$E$10</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$9</f>
+              <f>'실행이력'!$A$4:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$9</f>
+              <f>'실행이력'!$F$4:$F$10</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$9</f>
+              <f>'실행이력'!$A$4:$A$10</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$9</f>
+              <f>'실행이력'!$G$4:$G$10</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14559,6 +14559,48 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-03 02:57</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>fix/tracker-cache-bust</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>dd69cfb</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E10" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F10" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="35" t="n">
+        <v>294</v>
+      </c>
+      <c r="J10" s="35" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="K10" s="36">
+        <f>IFERROR(E10/(E10+F10+G10),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/aws-deploy, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$10</f>
+              <f>'실행이력'!$A$4:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$10</f>
+              <f>'실행이력'!$E$4:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$10</f>
+              <f>'실행이력'!$A$4:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$10</f>
+              <f>'실행이력'!$F$4:$F$11</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$10</f>
+              <f>'실행이력'!$A$4:$A$11</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$10</f>
+              <f>'실행이력'!$G$4:$G$11</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14601,6 +14601,48 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 16:11</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>feature/aws-deploy</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>f3f397a</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E11" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F11" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G11" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="35" t="n">
+        <v>308</v>
+      </c>
+      <c r="J11" s="35" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="K11" s="36">
+        <f>IFERROR(E11/(E11+F11+G11),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/https-budget, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$11</f>
+              <f>'실행이력'!$A$4:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$11</f>
+              <f>'실행이력'!$E$4:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$11</f>
+              <f>'실행이력'!$A$4:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$11</f>
+              <f>'실행이력'!$F$4:$F$12</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$11</f>
+              <f>'실행이력'!$A$4:$A$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$11</f>
+              <f>'실행이력'!$G$4:$G$12</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14643,6 +14643,48 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 17:11</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="inlineStr">
+        <is>
+          <t>feature/https-budget</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>1859e63</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E12" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F12" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G12" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="35" t="n">
+        <v>311</v>
+      </c>
+      <c r="J12" s="35" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="K12" s="36">
+        <f>IFERROR(E12/(E12+F12+G12),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/service-url, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$12</f>
+              <f>'실행이력'!$A$4:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$12</f>
+              <f>'실행이력'!$E$4:$E$13</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$12</f>
+              <f>'실행이력'!$A$4:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$12</f>
+              <f>'실행이력'!$F$4:$F$13</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$12</f>
+              <f>'실행이력'!$A$4:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$12</f>
+              <f>'실행이력'!$G$4:$G$13</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14685,6 +14685,48 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 17:29</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="inlineStr">
+        <is>
+          <t>feature/service-url</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>4b3607e</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E13" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F13" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G13" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="35" t="n">
+        <v>311</v>
+      </c>
+      <c r="J13" s="35" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="K13" s="36">
+        <f>IFERROR(E13/(E13+F13+G13),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/case-detail, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$13</f>
+              <f>'실행이력'!$A$4:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$13</f>
+              <f>'실행이력'!$E$4:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$13</f>
+              <f>'실행이력'!$A$4:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$13</f>
+              <f>'실행이력'!$F$4:$F$14</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$13</f>
+              <f>'실행이력'!$A$4:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$13</f>
+              <f>'실행이력'!$G$4:$G$14</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14727,6 +14727,48 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:29</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>feature/case-detail</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>e1f086b</t>
+        </is>
+      </c>
+      <c r="D14" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E14" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F14" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="35" t="n">
+        <v>312</v>
+      </c>
+      <c r="J14" s="35" t="n">
+        <v>27</v>
+      </c>
+      <c r="K14" s="36">
+        <f>IFERROR(E14/(E14+F14+G14),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/case-detail-prerun, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$14</f>
+              <f>'실행이력'!$A$4:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$14</f>
+              <f>'실행이력'!$E$4:$E$15</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$14</f>
+              <f>'실행이력'!$A$4:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$14</f>
+              <f>'실행이력'!$F$4:$F$15</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$14</f>
+              <f>'실행이력'!$A$4:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$14</f>
+              <f>'실행이력'!$G$4:$G$15</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14769,6 +14769,48 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:32</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="inlineStr">
+        <is>
+          <t>feature/case-detail-prerun</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>811f445</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E15" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G15" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="35" t="n">
+        <v>312</v>
+      </c>
+      <c r="J15" s="35" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="K15" s="36">
+        <f>IFERROR(E15/(E15+F15+G15),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/detail-layout, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$15</f>
+              <f>'실행이력'!$A$4:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$15</f>
+              <f>'실행이력'!$E$4:$E$16</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$15</f>
+              <f>'실행이력'!$A$4:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$15</f>
+              <f>'실행이력'!$F$4:$F$16</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$15</f>
+              <f>'실행이력'!$A$4:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$15</f>
+              <f>'실행이력'!$G$4:$G$16</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14811,6 +14811,48 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:42</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t>fix/detail-layout</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="inlineStr">
+        <is>
+          <t>d6dc555</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E16" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F16" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G16" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="35" t="n">
+        <v>312</v>
+      </c>
+      <c r="J16" s="35" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="K16" s="36">
+        <f>IFERROR(E16/(E16+F16+G16),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/demo-deploy-files, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$16</f>
+              <f>'실행이력'!$A$4:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$16</f>
+              <f>'실행이력'!$E$4:$E$17</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$16</f>
+              <f>'실행이력'!$A$4:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$16</f>
+              <f>'실행이력'!$F$4:$F$17</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$16</f>
+              <f>'실행이력'!$A$4:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$16</f>
+              <f>'실행이력'!$G$4:$G$17</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14853,6 +14853,48 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:43</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t>fix/demo-deploy-files</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>7d6b8d9</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E17" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F17" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G17" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="35" t="n">
+        <v>313</v>
+      </c>
+      <c r="J17" s="35" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="K17" s="36">
+        <f>IFERROR(E17/(E17+F17+G17),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/lazy-case-info, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$17</f>
+              <f>'실행이력'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$17</f>
+              <f>'실행이력'!$E$4:$E$18</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$17</f>
+              <f>'실행이력'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$17</f>
+              <f>'실행이력'!$F$4:$F$18</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$17</f>
+              <f>'실행이력'!$A$4:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$17</f>
+              <f>'실행이력'!$G$4:$G$18</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14895,6 +14895,48 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:47</t>
+        </is>
+      </c>
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t>fix/lazy-case-info</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>4df1cfb</t>
+        </is>
+      </c>
+      <c r="D18" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F18" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G18" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="35" t="n">
+        <v>314</v>
+      </c>
+      <c r="J18" s="35" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="K18" s="36">
+        <f>IFERROR(E18/(E18+F18+G18),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/run-one-case, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$18</f>
+              <f>'실행이력'!$A$4:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$18</f>
+              <f>'실행이력'!$E$4:$E$19</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$18</f>
+              <f>'실행이력'!$A$4:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$18</f>
+              <f>'실행이력'!$F$4:$F$19</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$18</f>
+              <f>'실행이력'!$A$4:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$18</f>
+              <f>'실행이력'!$G$4:$G$19</f>
             </numRef>
           </val>
         </ser>
@@ -14220,7 +14220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14937,6 +14937,48 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-11 23:58</t>
+        </is>
+      </c>
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t>feature/run-one-case</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>fb4a312</t>
+        </is>
+      </c>
+      <c r="D19" s="35" t="n">
+        <v>158</v>
+      </c>
+      <c r="E19" s="35" t="n">
+        <v>66</v>
+      </c>
+      <c r="F19" s="35" t="n">
+        <v>92</v>
+      </c>
+      <c r="G19" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="35" t="n">
+        <v>317</v>
+      </c>
+      <c r="J19" s="35" t="n">
+        <v>27</v>
+      </c>
+      <c r="K19" s="36">
+        <f>IFERROR(E19/(E19+F19+G19),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/weekly-report, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$22</f>
+              <f>'실행이력'!$A$4:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$22</f>
+              <f>'실행이력'!$E$4:$E$23</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$22</f>
+              <f>'실행이력'!$A$4:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$22</f>
+              <f>'실행이력'!$F$4:$F$23</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$22</f>
+              <f>'실행이력'!$A$4:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$22</f>
+              <f>'실행이력'!$G$4:$G$23</f>
             </numRef>
           </val>
         </ser>
@@ -17145,7 +17145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18030,6 +18030,48 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-26 00:31</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="inlineStr">
+        <is>
+          <t>feature/weekly-report</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="inlineStr">
+        <is>
+          <t>8a83a7e</t>
+        </is>
+      </c>
+      <c r="D23" s="35" t="n">
+        <v>197</v>
+      </c>
+      <c r="E23" s="35" t="n">
+        <v>132</v>
+      </c>
+      <c r="F23" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="G23" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="35" t="n">
+        <v>373</v>
+      </c>
+      <c r="J23" s="35" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="K23" s="36">
+        <f>IFERROR(E23/(E23+F23+G23),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/aws-lowcost, 테스트 failure)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$23</f>
+              <f>'실행이력'!$A$4:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$23</f>
+              <f>'실행이력'!$E$4:$E$24</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$23</f>
+              <f>'실행이력'!$A$4:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$23</f>
+              <f>'실행이력'!$F$4:$F$24</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$23</f>
+              <f>'실행이력'!$A$4:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$23</f>
+              <f>'실행이력'!$G$4:$G$24</f>
             </numRef>
           </val>
         </ser>
@@ -17145,7 +17145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18072,6 +18072,48 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-27 17:30</t>
+        </is>
+      </c>
+      <c r="B24" s="34" t="inlineStr">
+        <is>
+          <t>feature/aws-lowcost</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>b80b869</t>
+        </is>
+      </c>
+      <c r="D24" s="35" t="n">
+        <v>197</v>
+      </c>
+      <c r="E24" s="35" t="n">
+        <v>132</v>
+      </c>
+      <c r="F24" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="G24" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="35" t="n">
+        <v>373</v>
+      </c>
+      <c r="J24" s="35" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="K24" s="36">
+        <f>IFERROR(E24/(E24+F24+G24),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/dynamo-store, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$25</f>
+              <f>'실행이력'!$A$4:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$25</f>
+              <f>'실행이력'!$E$4:$E$26</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$25</f>
+              <f>'실행이력'!$A$4:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$25</f>
+              <f>'실행이력'!$F$4:$F$26</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$25</f>
+              <f>'실행이력'!$A$4:$A$26</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$25</f>
+              <f>'실행이력'!$G$4:$G$26</f>
             </numRef>
           </val>
         </ser>
@@ -17520,7 +17520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18531,6 +18531,48 @@
         <v/>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-27 18:26</t>
+        </is>
+      </c>
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>feature/dynamo-store</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>0f208f8</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="n">
+        <v>202</v>
+      </c>
+      <c r="E26" s="35" t="n">
+        <v>137</v>
+      </c>
+      <c r="F26" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="G26" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="35" t="n">
+        <v>430</v>
+      </c>
+      <c r="J26" s="35" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="K26" s="36">
+        <f>IFERROR(E26/(E26+F26+G26),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/lambda-deploy, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$26</f>
+              <f>'실행이력'!$A$4:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$26</f>
+              <f>'실행이력'!$E$4:$E$27</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$26</f>
+              <f>'실행이력'!$A$4:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$26</f>
+              <f>'실행이력'!$F$4:$F$27</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$26</f>
+              <f>'실행이력'!$A$4:$A$27</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$26</f>
+              <f>'실행이력'!$G$4:$G$27</f>
             </numRef>
           </val>
         </ser>
@@ -17520,7 +17520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18573,6 +18573,48 @@
         <v/>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-27 18:42</t>
+        </is>
+      </c>
+      <c r="B27" s="34" t="inlineStr">
+        <is>
+          <t>feature/lambda-deploy</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>8b6f0be</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="n">
+        <v>202</v>
+      </c>
+      <c r="E27" s="35" t="n">
+        <v>137</v>
+      </c>
+      <c r="F27" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="G27" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="35" t="n">
+        <v>433</v>
+      </c>
+      <c r="J27" s="35" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="K27" s="36">
+        <f>IFERROR(E27/(E27+F27+G27),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (fix/deploy-doc-policy, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$27</f>
+              <f>'실행이력'!$A$4:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$27</f>
+              <f>'실행이력'!$E$4:$E$28</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$27</f>
+              <f>'실행이력'!$A$4:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$27</f>
+              <f>'실행이력'!$F$4:$F$28</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$27</f>
+              <f>'실행이력'!$A$4:$A$28</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$27</f>
+              <f>'실행이력'!$G$4:$G$28</f>
             </numRef>
           </val>
         </ser>
@@ -17520,7 +17520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -18615,6 +18615,48 @@
         <v/>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-27 19:13</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="inlineStr">
+        <is>
+          <t>fix/deploy-doc-policy</t>
+        </is>
+      </c>
+      <c r="C28" s="33" t="inlineStr">
+        <is>
+          <t>23d9262</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="n">
+        <v>202</v>
+      </c>
+      <c r="E28" s="35" t="n">
+        <v>137</v>
+      </c>
+      <c r="F28" s="35" t="n">
+        <v>65</v>
+      </c>
+      <c r="G28" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="35" t="n">
+        <v>433</v>
+      </c>
+      <c r="J28" s="35" t="n">
+        <v>71</v>
+      </c>
+      <c r="K28" s="36">
+        <f>IFERROR(E28/(E28+F28+G28),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
chore: 시험 진척도 갱신 (feature/sc06-certs, 테스트 success)
</commit_message>
<xml_diff>
--- a/assets/tracker/test-tracker.xlsx
+++ b/assets/tracker/test-tracker.xlsx
@@ -721,12 +721,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$30</f>
+              <f>'실행이력'!$A$4:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$E$4:$E$30</f>
+              <f>'실행이력'!$E$4:$E$31</f>
             </numRef>
           </val>
         </ser>
@@ -763,12 +763,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$30</f>
+              <f>'실행이력'!$A$4:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$F$4:$F$30</f>
+              <f>'실행이력'!$F$4:$F$31</f>
             </numRef>
           </val>
         </ser>
@@ -805,12 +805,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'실행이력'!$A$4:$A$30</f>
+              <f>'실행이력'!$A$4:$A$31</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'실행이력'!$G$4:$G$30</f>
+              <f>'실행이력'!$G$4:$G$31</f>
             </numRef>
           </val>
         </ser>
@@ -14172,10 +14172,10 @@
         <v/>
       </c>
       <c r="D30" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" s="23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="23" t="n">
         <v>0</v>
@@ -14183,11 +14183,7 @@
       <c r="G30" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H30" s="22" t="inlineStr">
-        <is>
-          <t>AssertionError: assert '' != ''</t>
-        </is>
-      </c>
+      <c r="H30" s="22" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="22" t="inlineStr">
@@ -20070,7 +20066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21291,6 +21287,48 @@
         <v/>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>2026-10-31 21:03</t>
+        </is>
+      </c>
+      <c r="B31" s="34" t="inlineStr">
+        <is>
+          <t>feature/sc06-certs</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
+          <t>4ed2099</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="n">
+        <v>236</v>
+      </c>
+      <c r="E31" s="35" t="n">
+        <v>229</v>
+      </c>
+      <c r="F31" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="G31" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="35" t="n">
+        <v>532</v>
+      </c>
+      <c r="J31" s="35" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="K31" s="36">
+        <f>IFERROR(E31/(E31+F31+G31),0)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="K4:K600">
     <cfRule type="dataBar" priority="1">

</xml_diff>